<commit_message>
Match limits by method and country, fix Confluence header detection
- Match ticket `method` (then method without currency code, then
  subagent) against the Confluence "Метод" column; narrow candidates by
  ticket country via table heading / "Страна" column (EN<->RU aliases).
- Prefer the longest whole-word name on substring matches.
- Detect header rows built from <td> cells and skip repeated headers;
  ignore Переключалка / Страна / Доп.информация columns for limits.
- Default amount field to `amount` (Amount by receipt).
- Report Method, Confluence row country and country-match flag in UI
  and Excel; summary grouped by method + country.
- Diagnostics: per-ticket match check for Credited (M) tickets on page 1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BtxWwzwrUnpobVqxjUHajj
</commit_message>
<xml_diff>
--- a/out.xlsx
+++ b/out.xlsx
@@ -9,10 +9,10 @@
     <sheet name="Сводка" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Ниже лимита'!A1:N4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Выше лимита'!A1:N3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Не удалось проверить'!A1:I3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3">'Сводка'!A1:F4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Ниже лимита'!A1:P4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Выше лимита'!A1:P3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Не удалось проверить'!A1:J3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3">'Сводка'!A1:G4</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -613,22 +613,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:P4"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="19.83203125" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="19.83203125" customWidth="1"/>
     <col min="6" max="6" width="8.83203125" customWidth="1"/>
     <col min="7" max="7" width="8.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="9.83203125" customWidth="1"/>
-    <col min="10" max="10" width="11.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="21.83203125" customWidth="1"/>
-    <col min="13" max="13" width="19.83203125" customWidth="1"/>
-    <col min="14" max="14" width="38.83203125" customWidth="1"/>
+    <col min="8" max="8" width="8.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="9.83203125" customWidth="1"/>
+    <col min="11" max="11" width="11.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1"/>
+    <col min="14" max="14" width="21.83203125" customWidth="1"/>
+    <col min="15" max="15" width="16.83203125" customWidth="1"/>
+    <col min="16" max="16" width="38.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -639,39 +641,45 @@
         <v>Ticket ID</v>
       </c>
       <c r="C1" s="3" t="str">
+        <v>Method</v>
+      </c>
+      <c r="D1" s="3" t="str">
         <v>Subagent</v>
       </c>
-      <c r="D1" s="3" t="str">
+      <c r="E1" s="3" t="str">
         <v>Amount by receipt</v>
       </c>
-      <c r="E1" s="3" t="str">
+      <c r="F1" s="3" t="str">
         <v>Валюта</v>
       </c>
-      <c r="F1" s="3" t="str">
+      <c r="G1" s="3" t="str">
         <v>Min</v>
       </c>
-      <c r="G1" s="3" t="str">
+      <c r="H1" s="3" t="str">
         <v>Max</v>
       </c>
-      <c r="H1" s="3" t="str">
+      <c r="I1" s="3" t="str">
         <v>Отклонение</v>
       </c>
-      <c r="I1" s="3" t="str">
+      <c r="J1" s="3" t="str">
         <v>Country</v>
       </c>
-      <c r="J1" s="3" t="str">
+      <c r="K1" s="3" t="str">
         <v>User ID</v>
       </c>
-      <c r="K1" s="3" t="str">
+      <c r="L1" s="3" t="str">
         <v>Status</v>
       </c>
-      <c r="L1" s="3" t="str">
-        <v>Строка в Confluence</v>
-      </c>
       <c r="M1" s="3" t="str">
-        <v>Раздел Confluence</v>
+        <v>Метод в Confluence</v>
       </c>
       <c r="N1" s="3" t="str">
+        <v>Страна (Confluence)</v>
+      </c>
+      <c r="O1" s="3" t="str">
+        <v>Страна совпала</v>
+      </c>
+      <c r="P1" s="3" t="str">
         <v>Лимит (как в Confluence)</v>
       </c>
     </row>
@@ -683,39 +691,45 @@
         <v>1000001</v>
       </c>
       <c r="C2" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D2" s="4" t="str">
         <v>Vodafone Cash</v>
       </c>
-      <c r="D2" s="5">
+      <c r="E2" s="5">
         <v>50</v>
       </c>
-      <c r="E2" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F2" s="5">
+      <c r="F2" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G2" s="5">
         <v>100</v>
       </c>
-      <c r="G2" s="5">
+      <c r="H2" s="5">
         <v>5000</v>
       </c>
-      <c r="H2" s="5">
+      <c r="I2" s="5">
         <v>-50</v>
       </c>
-      <c r="I2" s="4" t="str">
+      <c r="J2" s="4" t="str">
         <v>Egypt</v>
       </c>
-      <c r="J2" s="4" t="str">
+      <c r="K2" s="4" t="str">
         <v>551000001</v>
       </c>
-      <c r="K2" s="4" t="str">
+      <c r="L2" s="4" t="str">
         <v>Credited (M)</v>
       </c>
-      <c r="L2" s="4" t="str">
+      <c r="M2" s="4" t="str">
         <v>Vodafone Cash</v>
       </c>
-      <c r="M2" s="4" t="str">
+      <c r="N2" s="4" t="str">
         <v>Egypt</v>
       </c>
-      <c r="N2" s="6" t="str">
+      <c r="O2" s="4" t="str">
+        <v>да</v>
+      </c>
+      <c r="P2" s="6" t="str">
         <v>от 100 до 5 000 EGP | звонить 2 раза</v>
       </c>
     </row>
@@ -727,39 +741,45 @@
         <v>1000005</v>
       </c>
       <c r="C3" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D3" s="4" t="str">
         <v>InstaPay</v>
       </c>
-      <c r="D3" s="5">
+      <c r="E3" s="5">
         <v>5</v>
       </c>
-      <c r="E3" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F3" s="5">
+      <c r="F3" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G3" s="5">
         <v>50</v>
       </c>
-      <c r="G3" s="5">
+      <c r="H3" s="5">
         <v>1000</v>
       </c>
-      <c r="H3" s="5">
+      <c r="I3" s="5">
         <v>-45</v>
       </c>
-      <c r="I3" s="4" t="str">
+      <c r="J3" s="4" t="str">
         <v>Egypt</v>
       </c>
-      <c r="J3" s="4" t="str">
+      <c r="K3" s="4" t="str">
         <v>551000005</v>
       </c>
-      <c r="K3" s="4" t="str">
+      <c r="L3" s="4" t="str">
         <v>207 - Credited (M)</v>
       </c>
-      <c r="L3" s="4" t="str">
+      <c r="M3" s="4" t="str">
         <v>InstaPay</v>
       </c>
-      <c r="M3" s="4" t="str">
+      <c r="N3" s="4" t="str">
         <v>Egypt</v>
       </c>
-      <c r="N3" s="6" t="str">
+      <c r="O3" s="4" t="str">
+        <v>да</v>
+      </c>
+      <c r="P3" s="6" t="str">
         <v>50 - 1000</v>
       </c>
     </row>
@@ -771,68 +791,76 @@
         <v>1000009</v>
       </c>
       <c r="C4" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D4" s="4" t="str">
         <v>Orange Money</v>
       </c>
-      <c r="D4" s="5">
+      <c r="E4" s="5">
         <v>1</v>
       </c>
-      <c r="E4" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F4" s="5">
+      <c r="F4" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G4" s="5">
         <v>10</v>
       </c>
-      <c r="G4" s="5">
+      <c r="H4" s="5">
         <v>1500</v>
       </c>
-      <c r="H4" s="5">
+      <c r="I4" s="5">
         <v>-9</v>
       </c>
-      <c r="I4" s="4" t="str">
+      <c r="J4" s="4" t="str">
         <v>Egypt</v>
       </c>
-      <c r="J4" s="4" t="str">
-        <v/>
-      </c>
       <c r="K4" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L4" s="4" t="str">
         <v>Credited (M)</v>
       </c>
-      <c r="L4" s="4" t="str">
+      <c r="M4" s="4" t="str">
         <v>Orange Money</v>
       </c>
-      <c r="M4" s="4" t="str">
+      <c r="N4" s="4" t="str">
         <v>Orange</v>
       </c>
-      <c r="N4" s="6" t="str">
+      <c r="O4" s="4" t="str">
+        <v>нет</v>
+      </c>
+      <c r="P4" s="6" t="str">
         <v>10 | 1 500</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N4"/>
+  <autoFilter ref="A1:P4"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:P3"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="19.83203125" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="19.83203125" customWidth="1"/>
     <col min="6" max="6" width="8.83203125" customWidth="1"/>
     <col min="7" max="7" width="8.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="9.83203125" customWidth="1"/>
-    <col min="10" max="10" width="11.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
-    <col min="12" max="12" width="21.83203125" customWidth="1"/>
-    <col min="13" max="13" width="19.83203125" customWidth="1"/>
-    <col min="14" max="14" width="38.83203125" customWidth="1"/>
+    <col min="8" max="8" width="8.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="9.83203125" customWidth="1"/>
+    <col min="11" max="11" width="11.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1"/>
+    <col min="14" max="14" width="21.83203125" customWidth="1"/>
+    <col min="15" max="15" width="16.83203125" customWidth="1"/>
+    <col min="16" max="16" width="38.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -843,39 +871,45 @@
         <v>Ticket ID</v>
       </c>
       <c r="C1" s="7" t="str">
+        <v>Method</v>
+      </c>
+      <c r="D1" s="7" t="str">
         <v>Subagent</v>
       </c>
-      <c r="D1" s="7" t="str">
+      <c r="E1" s="7" t="str">
         <v>Amount by receipt</v>
       </c>
-      <c r="E1" s="7" t="str">
+      <c r="F1" s="7" t="str">
         <v>Валюта</v>
       </c>
-      <c r="F1" s="7" t="str">
+      <c r="G1" s="7" t="str">
         <v>Min</v>
       </c>
-      <c r="G1" s="7" t="str">
+      <c r="H1" s="7" t="str">
         <v>Max</v>
       </c>
-      <c r="H1" s="7" t="str">
+      <c r="I1" s="7" t="str">
         <v>Отклонение</v>
       </c>
-      <c r="I1" s="7" t="str">
+      <c r="J1" s="7" t="str">
         <v>Country</v>
       </c>
-      <c r="J1" s="7" t="str">
+      <c r="K1" s="7" t="str">
         <v>User ID</v>
       </c>
-      <c r="K1" s="7" t="str">
+      <c r="L1" s="7" t="str">
         <v>Status</v>
       </c>
-      <c r="L1" s="7" t="str">
-        <v>Строка в Confluence</v>
-      </c>
       <c r="M1" s="7" t="str">
-        <v>Раздел Confluence</v>
+        <v>Метод в Confluence</v>
       </c>
       <c r="N1" s="7" t="str">
+        <v>Страна (Confluence)</v>
+      </c>
+      <c r="O1" s="7" t="str">
+        <v>Страна совпала</v>
+      </c>
+      <c r="P1" s="7" t="str">
         <v>Лимит (как в Confluence)</v>
       </c>
     </row>
@@ -887,39 +921,45 @@
         <v>1000002</v>
       </c>
       <c r="C2" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D2" s="4" t="str">
         <v>Vodafone Cash</v>
       </c>
-      <c r="D2" s="5">
-        <v>6000</v>
-      </c>
-      <c r="E2" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F2" s="5">
+      <c r="E2" s="5">
+        <v>9000</v>
+      </c>
+      <c r="F2" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G2" s="5">
         <v>100</v>
       </c>
-      <c r="G2" s="5">
+      <c r="H2" s="5">
         <v>5000</v>
       </c>
-      <c r="H2" s="5">
-        <v>1000</v>
-      </c>
-      <c r="I2" s="4" t="str">
+      <c r="I2" s="5">
+        <v>4000</v>
+      </c>
+      <c r="J2" s="4" t="str">
         <v>Egypt</v>
       </c>
-      <c r="J2" s="4" t="str">
+      <c r="K2" s="4" t="str">
         <v>551000002</v>
       </c>
-      <c r="K2" s="4" t="str">
+      <c r="L2" s="4" t="str">
         <v>Credited (M)</v>
       </c>
-      <c r="L2" s="4" t="str">
+      <c r="M2" s="4" t="str">
         <v>Vodafone Cash</v>
       </c>
-      <c r="M2" s="4" t="str">
+      <c r="N2" s="4" t="str">
         <v>Egypt</v>
       </c>
-      <c r="N2" s="6" t="str">
+      <c r="O2" s="4" t="str">
+        <v>да</v>
+      </c>
+      <c r="P2" s="6" t="str">
         <v>от 100 до 5 000 EGP | звонить 2 раза</v>
       </c>
     </row>
@@ -931,63 +971,70 @@
         <v>1000008</v>
       </c>
       <c r="C3" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D3" s="4" t="str">
         <v>Orange Money</v>
       </c>
-      <c r="D3" s="5">
+      <c r="E3" s="5">
         <v>2000</v>
       </c>
-      <c r="E3" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F3" s="5">
+      <c r="F3" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G3" s="5">
         <v>10</v>
       </c>
-      <c r="G3" s="5">
+      <c r="H3" s="5">
         <v>1500</v>
       </c>
-      <c r="H3" s="5">
+      <c r="I3" s="5">
         <v>500</v>
       </c>
-      <c r="I3" s="4" t="str">
+      <c r="J3" s="4" t="str">
         <v>Egypt</v>
       </c>
-      <c r="J3" s="4" t="str">
+      <c r="K3" s="4" t="str">
         <v>551000008</v>
       </c>
-      <c r="K3" s="4" t="str">
+      <c r="L3" s="4" t="str">
         <v>credited (m)</v>
       </c>
-      <c r="L3" s="4" t="str">
+      <c r="M3" s="4" t="str">
         <v>Orange Money</v>
       </c>
-      <c r="M3" s="4" t="str">
+      <c r="N3" s="4" t="str">
         <v>Orange</v>
       </c>
-      <c r="N3" s="6" t="str">
+      <c r="O3" s="4" t="str">
+        <v>нет</v>
+      </c>
+      <c r="P3" s="6" t="str">
         <v>10 | 1 500</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N3"/>
+  <autoFilter ref="A1:P3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="13.83203125" customWidth="1"/>
-    <col min="4" max="4" width="19.83203125" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" customWidth="1"/>
-    <col min="6" max="6" width="9.83203125" customWidth="1"/>
-    <col min="7" max="7" width="11.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="60.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="5" max="5" width="19.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="9.83203125" customWidth="1"/>
+    <col min="8" max="8" width="11.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -998,24 +1045,27 @@
         <v>Ticket ID</v>
       </c>
       <c r="C1" s="8" t="str">
+        <v>Method</v>
+      </c>
+      <c r="D1" s="8" t="str">
         <v>Subagent</v>
       </c>
-      <c r="D1" s="8" t="str">
+      <c r="E1" s="8" t="str">
         <v>Amount by receipt</v>
       </c>
-      <c r="E1" s="8" t="str">
+      <c r="F1" s="8" t="str">
         <v>Валюта</v>
       </c>
-      <c r="F1" s="8" t="str">
+      <c r="G1" s="8" t="str">
         <v>Country</v>
       </c>
-      <c r="G1" s="8" t="str">
+      <c r="H1" s="8" t="str">
         <v>User ID</v>
       </c>
-      <c r="H1" s="8" t="str">
+      <c r="I1" s="8" t="str">
         <v>Status</v>
       </c>
-      <c r="I1" s="8" t="str">
+      <c r="J1" s="8" t="str">
         <v>Причина</v>
       </c>
     </row>
@@ -1027,25 +1077,28 @@
         <v>1000006</v>
       </c>
       <c r="C2" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D2" s="4" t="str">
         <v>Unknown Sub</v>
       </c>
-      <c r="D2" s="5">
+      <c r="E2" s="5">
         <v>100</v>
       </c>
-      <c r="E2" s="4" t="str">
-        <v/>
-      </c>
       <c r="F2" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G2" s="4" t="str">
         <v>Egypt</v>
       </c>
-      <c r="G2" s="4" t="str">
+      <c r="H2" s="4" t="str">
         <v>551000006</v>
       </c>
-      <c r="H2" s="4" t="str">
+      <c r="I2" s="4" t="str">
         <v>Credited (M)</v>
       </c>
-      <c r="I2" s="6" t="str">
-        <v>субагент не найден в Confluence</v>
+      <c r="J2" s="6" t="str">
+        <v>метод не найден в Confluence</v>
       </c>
     </row>
     <row r="3">
@@ -1056,64 +1109,71 @@
         <v>1000007</v>
       </c>
       <c r="C3" s="4" t="str">
+        <v/>
+      </c>
+      <c r="D3" s="4" t="str">
         <v>Etisalat</v>
       </c>
-      <c r="D3" s="5">
+      <c r="E3" s="5">
         <v>100</v>
       </c>
-      <c r="E3" s="4" t="str">
-        <v/>
-      </c>
       <c r="F3" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G3" s="4" t="str">
         <v>Egypt</v>
       </c>
-      <c r="G3" s="4" t="str">
+      <c r="H3" s="4" t="str">
         <v>551000007</v>
       </c>
-      <c r="H3" s="4" t="str">
+      <c r="I3" s="4" t="str">
         <v>Credited (M)</v>
       </c>
-      <c r="I3" s="6" t="str">
-        <v>лимит в Confluence не распознан: «Etisalat» уточнять в чате</v>
+      <c r="J3" s="6" t="str">
+        <v>лимит в Confluence не распознан: «Etisalat» (Egypt) уточнять в чате</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I3"/>
+  <autoFilter ref="A1:J3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
-    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="9.83203125" customWidth="1"/>
     <col min="3" max="3" width="8.83203125" customWidth="1"/>
     <col min="4" max="4" width="8.83203125" customWidth="1"/>
     <col min="5" max="5" width="8.83203125" customWidth="1"/>
     <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="9" t="str">
-        <v>Subagent</v>
+        <v>Method</v>
       </c>
       <c r="B1" s="9" t="str">
+        <v>Country</v>
+      </c>
+      <c r="C1" s="9" t="str">
         <v>Ниже</v>
       </c>
-      <c r="C1" s="9" t="str">
+      <c r="D1" s="9" t="str">
         <v>Выше</v>
       </c>
-      <c r="D1" s="9" t="str">
+      <c r="E1" s="9" t="str">
         <v>Всего</v>
       </c>
-      <c r="E1" s="9" t="str">
+      <c r="F1" s="9" t="str">
         <v>Min</v>
       </c>
-      <c r="F1" s="9" t="str">
+      <c r="G1" s="9" t="str">
         <v>Max</v>
       </c>
     </row>
@@ -1121,19 +1181,22 @@
       <c r="A2" s="4" t="str">
         <v>Vodafone Cash</v>
       </c>
-      <c r="B2" s="4">
-        <v>1</v>
+      <c r="B2" s="4" t="str">
+        <v>Egypt</v>
       </c>
       <c r="C2" s="4">
         <v>1</v>
       </c>
       <c r="D2" s="4">
+        <v>1</v>
+      </c>
+      <c r="E2" s="4">
         <v>2</v>
       </c>
-      <c r="E2" s="5">
+      <c r="F2" s="5">
         <v>100</v>
       </c>
-      <c r="F2" s="10">
+      <c r="G2" s="10">
         <v>5000</v>
       </c>
     </row>
@@ -1141,19 +1204,22 @@
       <c r="A3" s="4" t="str">
         <v>Orange Money</v>
       </c>
-      <c r="B3" s="4">
-        <v>1</v>
+      <c r="B3" s="4" t="str">
+        <v>Egypt</v>
       </c>
       <c r="C3" s="4">
         <v>1</v>
       </c>
       <c r="D3" s="4">
+        <v>1</v>
+      </c>
+      <c r="E3" s="4">
         <v>2</v>
       </c>
-      <c r="E3" s="5">
+      <c r="F3" s="5">
         <v>10</v>
       </c>
-      <c r="F3" s="10">
+      <c r="G3" s="10">
         <v>1500</v>
       </c>
     </row>
@@ -1161,19 +1227,22 @@
       <c r="A4" s="4" t="str">
         <v>InstaPay</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="4" t="str">
+        <v>Egypt</v>
+      </c>
+      <c r="C4" s="4">
         <v>1</v>
       </c>
-      <c r="C4" s="4">
+      <c r="D4" s="4">
         <v>0</v>
       </c>
-      <c r="D4" s="4">
+      <c r="E4" s="4">
         <v>1</v>
       </c>
-      <c r="E4" s="5">
+      <c r="F4" s="5">
         <v>50</v>
       </c>
-      <c r="F4" s="10">
+      <c r="G4" s="10">
         <v>1000</v>
       </c>
     </row>
@@ -1182,7 +1251,7 @@
         <v>Сформировано</v>
       </c>
       <c r="B6" s="2" t="str">
-        <v>12.10.2026 10:26</v>
+        <v>12.10.2026 10:50</v>
       </c>
     </row>
     <row r="7">
@@ -1258,9 +1327,9 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
+  <autoFilter ref="A1:G4"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>